<commit_message>
Passage au Template 2 (#359)
* release 406

* Passage template2

---------

Co-authored-by: Nicolas Riss <48218773+nriss@users.noreply.github.com> 1be4c5661622d71659951c3628a23a32c7d8183d
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-input-task-sdo-codesystem.xlsx
+++ b/main/ig/CodeSystem-input-task-sdo-codesystem.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-23T16:16:52+00:00</t>
+    <t>2026-06-25T13:33:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>FRANCE</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>

<commit_message>
Preparation publication release 407 (#362) f235bf44fa67d1b9fba085ac066d0becc5590a39
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-input-task-sdo-codesystem.xlsx
+++ b/main/ig/CodeSystem-input-task-sdo-codesystem.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>4.0.6</t>
+    <t>4.0.7</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-26T14:37:44+00:00</t>
+    <t>2026-06-29T07:12:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>